<commit_message>
feat(base): complete modular base overhaul
</commit_message>
<xml_diff>
--- a/assets/registry/ShellStorm2_美术资产台账_v001.xlsx
+++ b/assets/registry/ShellStorm2_美术资产台账_v001.xlsx
@@ -2,24 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R0127ac44682d4feb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资产主表" sheetId="2" r:id="R7e1e467d3eb045cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="角色组件" sheetId="3" r:id="Rcf071e60b0814c5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="动画与状态" sheetId="4" r:id="Rf4c20de826454a01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类与编码" sheetId="5" r:id="R7da4dd0fe97f4e9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="命名与查重" sheetId="6" r:id="R0496e026e72a4888"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原型角色" sheetId="7" r:id="Rf80ac4b71a2d49ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="8" r:id="Rba66325e1ff6496c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D Prefab总控" sheetId="9" r:id="R35820ff189dd4719"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-场景通用" sheetId="10" r:id="R24ffccdbd22349b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-设施" sheetId="11" r:id="R6a70d1f70e76411c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-道具" sheetId="12" r:id="R116530e24c78471b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-角色" sheetId="13" r:id="R78d22c4d378b42e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-敌人" sheetId="14" r:id="R16db15341bda4c23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-武器" sheetId="15" r:id="Rba3ee9eef5ed43a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-物品" sheetId="16" r:id="R1e8880fac14749cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-特效" sheetId="17" r:id="R6b6ab662236848a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-其他" sheetId="18" r:id="Rb95333a1b9864b12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R111badf2faa4436f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资产主表" sheetId="2" r:id="Rf7216e33164d410c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="角色组件" sheetId="3" r:id="Rfa13bef7b1204d3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="动画与状态" sheetId="4" r:id="R34782d7f354d4ad7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类与编码" sheetId="5" r:id="Rb2f49475948646de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="命名与查重" sheetId="6" r:id="R0d1a957fa8294355"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原型角色" sheetId="7" r:id="R86ee98e9878f4cf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="8" r:id="R5b7fd96b0adc47c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D Prefab总控" sheetId="9" r:id="Re43a9b6df2714656"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-场景通用" sheetId="10" r:id="R2ee6d32d33184c32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-设施" sheetId="11" r:id="R4b1b60d4f0e7483d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-道具" sheetId="12" r:id="R810920693ae24707"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-角色" sheetId="13" r:id="R1511a47ea7da471f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-敌人" sheetId="14" r:id="Rcb69e40406de4a78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-武器" sheetId="15" r:id="R798ba1463c1c478a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-物品" sheetId="16" r:id="R258657c401384f9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-特效" sheetId="17" r:id="R4219a7cdcc414a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-其他" sheetId="18" r:id="Rfde33724019b4035"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skill清单" sheetId="19" r:id="R6e5bf74ed43240d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -214,7 +215,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="41">
+  <x:fills count="44">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -416,8 +417,23 @@
         <x:fgColor rgb="FFE2E8F0"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE6F1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F75B5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="40">
+  <x:borders count="41">
     <x:border/>
     <x:border>
       <x:left style="medium">
@@ -815,11 +831,25 @@
         <x:color rgb="FFD9E2F3"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF9FBAD0"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="333">
+  <x:cellXfs count="347">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -1607,6 +1637,34 @@
     <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="43" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="43" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="43" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="43" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="28" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2456,7 +2514,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="145" t="str">
-        <x:v>关卡结构、地板、墙体、走廊、楼梯、楼板与环境套件；当前 52 个独立Prefab。</x:v>
+        <x:v>关卡结构、地板、墙体、走廊、楼梯、楼板与环境套件；当前 55 个独立Prefab。</x:v>
       </x:c>
       <x:c r="B2" s="145"/>
       <x:c r="C2" s="145"/>
@@ -4970,6 +5028,156 @@
       </x:c>
       <x:c r="P56" t="str">
         <x:v>子Prefab=60；北墙两端普通+中间4窗；其余19普通墙，东侧1门墙；复用现有墙/地板资产，cast_and_receive；18米屋顶阻挡室外光；不恢复99/100层中间36块。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="78" customHeight="1">
+      <x:c r="A57" s="136" t="str">
+        <x:v>ENV-BASE99-MEZZANINE-20X10-Z5</x:v>
+      </x:c>
+      <x:c r="B57" s="136" t="str">
+        <x:v>基地99层5米楼中楼楼板</x:v>
+      </x:c>
+      <x:c r="C57" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/runtime/env_base99_mezzanine_20x10_z5/env_base99_mezzanine_20x10_z5_root_top3d_v002.tscn</x:v>
+      </x:c>
+      <x:c r="D57" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/components/env_base99_mezzanine_20x10_z5/env_base99_mezzanine_20x10_z5_visual_top3d_v002.glb</x:v>
+      </x:c>
+      <x:c r="E57" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/source/env_base99_modular_room/env_base99_modular_room_assets_clean_v002.blend</x:v>
+      </x:c>
+      <x:c r="F57" s="136" t="str">
+        <x:v>5米承重楼板；连续栏杆阻挡；真实投影</x:v>
+      </x:c>
+      <x:c r="G57" s="136" t="str">
+        <x:v>src/world3d/Base99WalkableModule3D.gd</x:v>
+      </x:c>
+      <x:c r="H57" s="136" t="str">
+        <x:v>开</x:v>
+      </x:c>
+      <x:c r="I57" s="136" t="str">
+        <x:v>Prefab自身</x:v>
+      </x:c>
+      <x:c r="J57" s="136" t="str">
+        <x:v>连续Box楼板+独立栏杆Box</x:v>
+      </x:c>
+      <x:c r="K57" s="136" t="str">
+        <x:v>20.2475×10.2475×5.93m；台面5m</x:v>
+      </x:c>
+      <x:c r="L57" s="136" t="str">
+        <x:v>底面中心；Blender -Y / Godot -Z</x:v>
+      </x:c>
+      <x:c r="M57" s="136" t="str">
+        <x:v>99层基地楼中楼</x:v>
+      </x:c>
+      <x:c r="N57" s="136" t="str">
+        <x:v>正式美术已接入</x:v>
+      </x:c>
+      <x:c r="O57" s="136" t="str">
+        <x:v>v002</x:v>
+      </x:c>
+      <x:c r="P57" s="136" t="str">
+        <x:v>根缩放1；替代Z7版本；视觉/碰撞/功能分离</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="78" customHeight="1">
+      <x:c r="A58" s="136" t="str">
+        <x:v>ENV-BASE99-STAIR-L-Z5</x:v>
+      </x:c>
+      <x:c r="B58" s="136" t="str">
+        <x:v>基地99层5米L型楼梯</x:v>
+      </x:c>
+      <x:c r="C58" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/runtime/env_base99_stair_l_z5/env_base99_stair_l_z5_root_top3d_v002.tscn</x:v>
+      </x:c>
+      <x:c r="D58" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/components/env_base99_stair_l_z5/env_base99_stair_l_z5_visual_top3d_v002.glb</x:v>
+      </x:c>
+      <x:c r="E58" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/source/env_base99_modular_room/env_base99_modular_room_assets_clean_v002.blend</x:v>
+      </x:c>
+      <x:c r="F58" s="136" t="str">
+        <x:v>0→2.5→5米双跑L梯；扶手真实投影与阻挡</x:v>
+      </x:c>
+      <x:c r="G58" s="136" t="str">
+        <x:v>src/world3d/Base99WalkableModule3D.gd</x:v>
+      </x:c>
+      <x:c r="H58" s="136" t="str">
+        <x:v>开</x:v>
+      </x:c>
+      <x:c r="I58" s="136" t="str">
+        <x:v>Prefab自身</x:v>
+      </x:c>
+      <x:c r="J58" s="136" t="str">
+        <x:v>两段连续斜坡+平台+独立扶手Box</x:v>
+      </x:c>
+      <x:c r="K58" s="136" t="str">
+        <x:v>9.2176×10.538×5.91015m；终点5m</x:v>
+      </x:c>
+      <x:c r="L58" s="136" t="str">
+        <x:v>底面中心；Blender -Y / Godot -Z</x:v>
+      </x:c>
+      <x:c r="M58" s="136" t="str">
+        <x:v>99层基地一楼至楼中楼</x:v>
+      </x:c>
+      <x:c r="N58" s="136" t="str">
+        <x:v>正式美术已接入</x:v>
+      </x:c>
+      <x:c r="O58" s="136" t="str">
+        <x:v>v002</x:v>
+      </x:c>
+      <x:c r="P58" s="136" t="str">
+        <x:v>不用逐级碰撞；坡脚/平台/坡顶连续；替代Z7版本</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="78" customHeight="1">
+      <x:c r="A59" s="136" t="str">
+        <x:v>ENV-BASE99-STAIR-EXTERIOR-H4</x:v>
+      </x:c>
+      <x:c r="B59" s="136" t="str">
+        <x:v>基地99至100层4米外门楼梯</x:v>
+      </x:c>
+      <x:c r="C59" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/runtime/env_base99_stair_exterior_h4/env_base99_stair_exterior_h4_root_top3d_v002.tscn</x:v>
+      </x:c>
+      <x:c r="D59" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/components/env_base99_stair_exterior_h4/env_base99_stair_exterior_h4_visual_top3d_v002.glb</x:v>
+      </x:c>
+      <x:c r="E59" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/source/env_base99_modular_room/env_base99_modular_room_assets_clean_v002.blend</x:v>
+      </x:c>
+      <x:c r="F59" s="136" t="str">
+        <x:v>平台5米至100层9米；两段原生楼梯组合；真实投影</x:v>
+      </x:c>
+      <x:c r="G59" s="136" t="str">
+        <x:v>src/world3d/Base99WalkableModule3D.gd</x:v>
+      </x:c>
+      <x:c r="H59" s="136" t="str">
+        <x:v>开</x:v>
+      </x:c>
+      <x:c r="I59" s="136" t="str">
+        <x:v>Prefab自身</x:v>
+      </x:c>
+      <x:c r="J59" s="136" t="str">
+        <x:v>覆盖8.515米包络的连续斜坡+双侧护栏</x:v>
+      </x:c>
+      <x:c r="K59" s="136" t="str">
+        <x:v>8.515×2.8×4m；高差4m</x:v>
+      </x:c>
+      <x:c r="L59" s="136" t="str">
+        <x:v>底面中心；Blender -Y / Godot -Z</x:v>
+      </x:c>
+      <x:c r="M59" s="136" t="str">
+        <x:v>基地楼中楼至100层出口</x:v>
+      </x:c>
+      <x:c r="N59" s="136" t="str">
+        <x:v>正式美术已接入</x:v>
+      </x:c>
+      <x:c r="O59" s="136" t="str">
+        <x:v>v002</x:v>
+      </x:c>
+      <x:c r="P59" s="136" t="str">
+        <x:v>不做纵向拉伸；替代H2版本</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5036,7 +5244,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="145" t="str">
-        <x:v>门扇、灯具、开关、终端、工作台、储物与服务设施；当前 15 个独立Prefab。</x:v>
+        <x:v>门扇、灯具、开关、终端、工作台、储物与服务设施；当前 17 个独立Prefab。</x:v>
       </x:c>
       <x:c r="B2" s="145"/>
       <x:c r="C2" s="145"/>
@@ -5834,6 +6042,102 @@
       </x:c>
       <x:c r="P19" s="136" t="str">
         <x:v>GLB无玩法碰撞；cast_and_receive；替换同路径GLB不改变门功能。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="78" customHeight="1">
+      <x:c r="A20" s="136" t="str">
+        <x:v>PRP-BASE-RECOVERY-STATION-3D</x:v>
+      </x:c>
+      <x:c r="B20" s="136" t="str">
+        <x:v>基地状态恢复舱</x:v>
+      </x:c>
+      <x:c r="C20" s="136" t="str">
+        <x:v>assets/art/props/base_world_3d/runtime/recovery_station/prp_base_recovery_station_root_top3d_v001.tscn</x:v>
+      </x:c>
+      <x:c r="D20" s="136"/>
+      <x:c r="E20" s="136"/>
+      <x:c r="F20" s="136" t="str">
+        <x:v>消耗基地电量恢复HP与手电电量</x:v>
+      </x:c>
+      <x:c r="G20" s="136" t="str">
+        <x:v>src/base3d/BaseFacility3D.gd; src/ui/BaseRecoveryMenu.gd; src/base/BaseEnergyService.gd</x:v>
+      </x:c>
+      <x:c r="H20" s="136" t="str">
+        <x:v>开</x:v>
+      </x:c>
+      <x:c r="I20" s="136" t="str">
+        <x:v>Prefab自身</x:v>
+      </x:c>
+      <x:c r="J20" s="136" t="str">
+        <x:v>Area3D交互+BoxShape3D实体</x:v>
+      </x:c>
+      <x:c r="K20" s="136" t="str">
+        <x:v>设施根缩放1；程序占位视觉</x:v>
+      </x:c>
+      <x:c r="L20" s="136" t="str">
+        <x:v>底面中心；-Z</x:v>
+      </x:c>
+      <x:c r="M20" s="136" t="str">
+        <x:v>BaseWorld3D/TowerDescent99F</x:v>
+      </x:c>
+      <x:c r="N20" s="136" t="str">
+        <x:v>功能已接入/正式模型待补</x:v>
+      </x:c>
+      <x:c r="O20" s="136" t="str">
+        <x:v>v001</x:v>
+      </x:c>
+      <x:c r="P20" s="136" t="str">
+        <x:v>手电在基地只暂停耗电；补电仅走恢复舱或电池</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="78" customHeight="1">
+      <x:c r="A21" s="136" t="str">
+        <x:v>PRP-BASE-AVATAR-WARDROBE-001</x:v>
+      </x:c>
+      <x:c r="B21" s="136" t="str">
+        <x:v>基地角色衣柜</x:v>
+      </x:c>
+      <x:c r="C21" s="136" t="str">
+        <x:v>assets/art/props/base_world_3d/runtime/avatar_wardrobe/prp_base_avatar_wardrobe_root_top3d_v001.tscn</x:v>
+      </x:c>
+      <x:c r="D21" s="136" t="str">
+        <x:v>assets/art/props/base_world_3d/components/locker_station/prp_base_locker_station_visual_top3d_v004.glb</x:v>
+      </x:c>
+      <x:c r="E21" s="136" t="str">
+        <x:v>assets/art/props/base_world_3d/source/locker_station/prp_base_locker_station_source_v004.blend</x:v>
+      </x:c>
+      <x:c r="F21" s="136" t="str">
+        <x:v>激活衣柜UI并预览/保存角色外观</x:v>
+      </x:c>
+      <x:c r="G21" s="136" t="str">
+        <x:v>src/base3d/wardrobe/WardrobeFacility3D.gd; src/ui/wardrobe/WardrobeMenu3D.gd</x:v>
+      </x:c>
+      <x:c r="H21" s="136" t="str">
+        <x:v>开</x:v>
+      </x:c>
+      <x:c r="I21" s="136" t="str">
+        <x:v>Prefab自身</x:v>
+      </x:c>
+      <x:c r="J21" s="136" t="str">
+        <x:v>Area3D交互+BoxShape3D实体；复用储物站视觉</x:v>
+      </x:c>
+      <x:c r="K21" s="136" t="str">
+        <x:v>5×3.9×1.63m碰撞；根缩放1</x:v>
+      </x:c>
+      <x:c r="L21" s="136" t="str">
+        <x:v>底面中心；-Z</x:v>
+      </x:c>
+      <x:c r="M21" s="136" t="str">
+        <x:v>BaseWorld3D/TowerDescent99F</x:v>
+      </x:c>
+      <x:c r="N21" s="136" t="str">
+        <x:v>功能已接入/复用模型</x:v>
+      </x:c>
+      <x:c r="O21" s="136" t="str">
+        <x:v>v001</x:v>
+      </x:c>
+      <x:c r="P21" s="136" t="str">
+        <x:v>6类方形物品格；每类≥3款；只改表现，不改碰撞与功能</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6174,7 +6478,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="250" t="str">
-        <x:v>玩家、NPC与角色表现/玩法根；本次扫描 3 个独立Prefab。</x:v>
+        <x:v>玩家、NPC与角色表现/玩法根及制作母版；当前 4 个登记项。</x:v>
       </x:c>
       <x:c r="B2" s="250"/>
       <x:c r="C2" s="250"/>
@@ -6380,6 +6684,52 @@
       </x:c>
       <x:c r="P7" s="196" t="str">
         <x:v>根节点=Player3D(CharacterBody3D)；子Prefab=2；资产主表当前Prefab=assets/art/characters/player/chr_player_capsule01_3d/variants/bunny01/chr_player_capsule01_bunny01_root_top3d_v006.tscn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="78" customHeight="1">
+      <x:c r="A8" s="136" t="str">
+        <x:v>CHR-PLAYER-AVATAR-TEMPLATE-001</x:v>
+      </x:c>
+      <x:c r="B8" s="136" t="str">
+        <x:v>玩家角色1.5米Blender制作母版</x:v>
+      </x:c>
+      <x:c r="C8" s="136"/>
+      <x:c r="D8" s="136"/>
+      <x:c r="E8" s="136" t="str">
+        <x:v>assets/art/characters/player/chr_player_avatar_template_3d/source/chr_player_avatar_template_source_v001.blend</x:v>
+      </x:c>
+      <x:c r="F8" s="136" t="str">
+        <x:v>角色与配件制作尺寸/方向/挂点模板；非运行时Prefab</x:v>
+      </x:c>
+      <x:c r="G8" s="136" t="str">
+        <x:v>scripts/blender/validate_player_avatar_asset_template.py</x:v>
+      </x:c>
+      <x:c r="H8" s="136" t="str">
+        <x:v>无</x:v>
+      </x:c>
+      <x:c r="I8" s="136" t="str">
+        <x:v>Player3D玩法根</x:v>
+      </x:c>
+      <x:c r="J8" s="136" t="str">
+        <x:v>母版只提供表现包络与挂点；CapsuleShape3D不变</x:v>
+      </x:c>
+      <x:c r="K8" s="136" t="str">
+        <x:v>总高1.50m；根缩放1</x:v>
+      </x:c>
+      <x:c r="L8" s="136" t="str">
+        <x:v>脚底中心Z0；Blender -Y / Godot -Z</x:v>
+      </x:c>
+      <x:c r="M8" s="136" t="str">
+        <x:v>玩家角色与换装资产制作</x:v>
+      </x:c>
+      <x:c r="N8" s="136" t="str">
+        <x:v>正式制作母版</x:v>
+      </x:c>
+      <x:c r="O8" s="136" t="str">
+        <x:v>v001</x:v>
+      </x:c>
+      <x:c r="P8" s="136" t="str">
+        <x:v>7槽位/9挂点；角色玩法碰撞仍由scenes/Player3D.tscn拥有</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8330,6 +8680,219 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="58" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="335" t="str">
+        <x:v>ShellStorm2 · 资产制作与带入 Skill 清单</x:v>
+      </x:c>
+      <x:c r="B1" s="335"/>
+      <x:c r="C1" s="335"/>
+      <x:c r="D1" s="335"/>
+      <x:c r="E1" s="335"/>
+      <x:c r="F1" s="335"/>
+      <x:c r="G1" s="335"/>
+      <x:c r="H1" s="335"/>
+      <x:c r="I1" s="335"/>
+      <x:c r="J1" s="335"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="338" t="str">
+        <x:v>只登记实际使用或项目预备的Skill；项目草稿不等于已安装。</x:v>
+      </x:c>
+      <x:c r="B2" s="338"/>
+      <x:c r="C2" s="338"/>
+      <x:c r="D2" s="338"/>
+      <x:c r="E2" s="338"/>
+      <x:c r="F2" s="338"/>
+      <x:c r="G2" s="338"/>
+      <x:c r="H2" s="338"/>
+      <x:c r="I2" s="338"/>
+      <x:c r="J2" s="338"/>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="344" t="str">
+        <x:v>SkillID</x:v>
+      </x:c>
+      <x:c r="B4" s="344" t="str">
+        <x:v>名称</x:v>
+      </x:c>
+      <x:c r="C4" s="344" t="str">
+        <x:v>用途</x:v>
+      </x:c>
+      <x:c r="D4" s="344" t="str">
+        <x:v>路径</x:v>
+      </x:c>
+      <x:c r="E4" s="344" t="str">
+        <x:v>安装状态</x:v>
+      </x:c>
+      <x:c r="F4" s="344" t="str">
+        <x:v>触发范围</x:v>
+      </x:c>
+      <x:c r="G4" s="344" t="str">
+        <x:v>版本</x:v>
+      </x:c>
+      <x:c r="H4" s="344" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+      <x:c r="I4" s="344" t="str">
+        <x:v>更新时间</x:v>
+      </x:c>
+      <x:c r="J4" s="344" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="56" customHeight="1">
+      <x:c r="A5" s="345" t="str">
+        <x:v>SKILL-SHELLSTORM-ART-ASSETS</x:v>
+      </x:c>
+      <x:c r="B5" s="345" t="str">
+        <x:v>ShellStorm2美术资产管理</x:v>
+      </x:c>
+      <x:c r="C5" s="345" t="str">
+        <x:v>资产分类、命名、查重、登记与QA</x:v>
+      </x:c>
+      <x:c r="D5" s="345" t="str">
+        <x:v>/Users/summercards/.codex/skills/shellstorm-art-assets/SKILL.md</x:v>
+      </x:c>
+      <x:c r="E5" s="345" t="str">
+        <x:v>已安装</x:v>
+      </x:c>
+      <x:c r="F5" s="345" t="str">
+        <x:v>ShellStorm2全类别美术资产</x:v>
+      </x:c>
+      <x:c r="G5" s="345" t="str">
+        <x:v>current</x:v>
+      </x:c>
+      <x:c r="H5" s="345" t="str">
+        <x:v>使用中</x:v>
+      </x:c>
+      <x:c r="I5" s="346" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="J5" s="345" t="str">
+        <x:v>项目资产总流程</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="56" customHeight="1">
+      <x:c r="A6" s="345" t="str">
+        <x:v>SKILL-BLENDER-GAME-PROP</x:v>
+      </x:c>
+      <x:c r="B6" s="345" t="str">
+        <x:v>Blender游戏资产制作规范</x:v>
+      </x:c>
+      <x:c r="C6" s="345" t="str">
+        <x:v>单物件与模块化建筑制作/验收</x:v>
+      </x:c>
+      <x:c r="D6" s="345" t="str">
+        <x:v>.codex/skills/blender-game-prop-standard/SKILL.md</x:v>
+      </x:c>
+      <x:c r="E6" s="345" t="str">
+        <x:v>项目内已安装</x:v>
+      </x:c>
+      <x:c r="F6" s="345" t="str">
+        <x:v>设施、道具、墙、楼板、楼梯、栏杆</x:v>
+      </x:c>
+      <x:c r="G6" s="345" t="str">
+        <x:v>current</x:v>
+      </x:c>
+      <x:c r="H6" s="345" t="str">
+        <x:v>本轮已迭代</x:v>
+      </x:c>
+      <x:c r="I6" s="346" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="J6" s="345" t="str">
+        <x:v>新增连接模块、高度、坡面、栏杆和投影规则</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="56" customHeight="1">
+      <x:c r="A7" s="345" t="str">
+        <x:v>SKILL-GODOT-MODEL-IMPORT</x:v>
+      </x:c>
+      <x:c r="B7" s="345" t="str">
+        <x:v>Godot模型资产导入规范</x:v>
+      </x:c>
+      <x:c r="C7" s="345" t="str">
+        <x:v>GLB、PackedScene、引用替换、台账和验收</x:v>
+      </x:c>
+      <x:c r="D7" s="345" t="str">
+        <x:v>.codex/skills/godot-model-asset-import-standard/SKILL.md</x:v>
+      </x:c>
+      <x:c r="E7" s="345" t="str">
+        <x:v>项目内已安装</x:v>
+      </x:c>
+      <x:c r="F7" s="345" t="str">
+        <x:v>所有3D模型导入与替换</x:v>
+      </x:c>
+      <x:c r="G7" s="345" t="str">
+        <x:v>current</x:v>
+      </x:c>
+      <x:c r="H7" s="345" t="str">
+        <x:v>本轮已迭代</x:v>
+      </x:c>
+      <x:c r="I7" s="346" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="J7" s="345" t="str">
+        <x:v>新增Prefab台账、结构碰撞和物理楼层规则</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="56" customHeight="1">
+      <x:c r="A8" s="345" t="str">
+        <x:v>SKILL-PLAYER-AVATAR-DRAFT</x:v>
+      </x:c>
+      <x:c r="B8" s="345" t="str">
+        <x:v>玩家角色资产制作与带入规范</x:v>
+      </x:c>
+      <x:c r="C8" s="345" t="str">
+        <x:v>1.5米角色母版、槽位、挂点、换装与导入</x:v>
+      </x:c>
+      <x:c r="D8" s="345" t="str">
+        <x:v>skills_drafts/player-avatar-asset-standard/SKILL.md</x:v>
+      </x:c>
+      <x:c r="E8" s="345" t="str">
+        <x:v>未安装（项目草稿）</x:v>
+      </x:c>
+      <x:c r="F8" s="345" t="str">
+        <x:v>玩家角色与配件</x:v>
+      </x:c>
+      <x:c r="G8" s="345" t="str">
+        <x:v>v001</x:v>
+      </x:c>
+      <x:c r="H8" s="345" t="str">
+        <x:v>预备完成</x:v>
+      </x:c>
+      <x:c r="I8" s="346" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="J8" s="345" t="str">
+        <x:v>等待用户未来明确授权后再安装</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -36838,6 +37401,446 @@
         <x:v>北墙两端普通+中间4窗；其余19普通墙，东侧1门墙；18米屋顶挡光；围护与封顶统一投影；不恢复99/100层中间36块。</x:v>
       </x:c>
     </x:row>
+    <x:row r="281" ht="66" customHeight="1">
+      <x:c r="A281" s="136" t="str">
+        <x:v>ENV-BASE99-MEZZANINE-20X10-Z5</x:v>
+      </x:c>
+      <x:c r="B281" s="136" t="str">
+        <x:v>基地99层5米楼中楼楼板</x:v>
+      </x:c>
+      <x:c r="C281" s="136" t="str">
+        <x:v>场景</x:v>
+      </x:c>
+      <x:c r="D281" s="136" t="str">
+        <x:v>environment_module</x:v>
+      </x:c>
+      <x:c r="E281" s="136" t="str">
+        <x:v>base99_mezzanine_20x10_z5</x:v>
+      </x:c>
+      <x:c r="F281" s="136" t="str">
+        <x:v>platform</x:v>
+      </x:c>
+      <x:c r="G281" s="136" t="str">
+        <x:v>ENV-BASE99-MODULAR-ROOM</x:v>
+      </x:c>
+      <x:c r="H281" s="136" t="str">
+        <x:v>俯视3D</x:v>
+      </x:c>
+      <x:c r="I281" s="136" t="str">
+        <x:v>default</x:v>
+      </x:c>
+      <x:c r="J281" s="136" t="str">
+        <x:v>基地99F</x:v>
+      </x:c>
+      <x:c r="K281" s="136" t="str">
+        <x:v>正式美术已接入</x:v>
+      </x:c>
+      <x:c r="L281" s="136" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="M281" s="136" t="str">
+        <x:v>v002</x:v>
+      </x:c>
+      <x:c r="N281" s="136" t="str">
+        <x:v>台面5m；20.2475×10.2475m</x:v>
+      </x:c>
+      <x:c r="O281" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/runtime/env_base99_mezzanine_20x10_z5/env_base99_mezzanine_20x10_z5_root_top3d_v002.tscn</x:v>
+      </x:c>
+      <x:c r="P281" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/source/env_base99_modular_room/env_base99_modular_room_assets_clean_v002.blend</x:v>
+      </x:c>
+      <x:c r="Q281" s="136" t="str">
+        <x:v>5米楼板; 栏杆; 投影</x:v>
+      </x:c>
+      <x:c r="R281" s="136" t="str">
+        <x:f>TEXTJOIN("|",TRUE,C281,D281,E281,F281,H281,I281)</x:f>
+        <x:v>场景|environment_module|base99_mezzanine_20x10_z5|platform|俯视3D|default</x:v>
+      </x:c>
+      <x:c r="S281" s="136" t="str">
+        <x:f>IF(COUNTIF($R$6:$R$400,R281)&gt;1,"重复","唯一")</x:f>
+        <x:v>唯一</x:v>
+      </x:c>
+      <x:c r="T281" s="136"/>
+      <x:c r="U281" s="136" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="V281" s="137" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="W281" s="136" t="str">
+        <x:v>用户自制/项目内资产</x:v>
+      </x:c>
+      <x:c r="X281" s="136" t="str">
+        <x:v>2026-08-20：本轮基地系统、角色母版与资产流程登记。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="282" ht="66" customHeight="1">
+      <x:c r="A282" s="136" t="str">
+        <x:v>ENV-BASE99-STAIR-L-Z5</x:v>
+      </x:c>
+      <x:c r="B282" s="136" t="str">
+        <x:v>基地99层5米L型楼梯</x:v>
+      </x:c>
+      <x:c r="C282" s="136" t="str">
+        <x:v>场景</x:v>
+      </x:c>
+      <x:c r="D282" s="136" t="str">
+        <x:v>environment_module</x:v>
+      </x:c>
+      <x:c r="E282" s="136" t="str">
+        <x:v>base99_stair_l_z5</x:v>
+      </x:c>
+      <x:c r="F282" s="136" t="str">
+        <x:v>stair</x:v>
+      </x:c>
+      <x:c r="G282" s="136" t="str">
+        <x:v>ENV-BASE99-MODULAR-ROOM</x:v>
+      </x:c>
+      <x:c r="H282" s="136" t="str">
+        <x:v>俯视3D</x:v>
+      </x:c>
+      <x:c r="I282" s="136" t="str">
+        <x:v>default</x:v>
+      </x:c>
+      <x:c r="J282" s="136" t="str">
+        <x:v>基地99F</x:v>
+      </x:c>
+      <x:c r="K282" s="136" t="str">
+        <x:v>正式美术已接入</x:v>
+      </x:c>
+      <x:c r="L282" s="136" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="M282" s="136" t="str">
+        <x:v>v002</x:v>
+      </x:c>
+      <x:c r="N282" s="136" t="str">
+        <x:v>0→2.5→5m</x:v>
+      </x:c>
+      <x:c r="O282" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/runtime/env_base99_stair_l_z5/env_base99_stair_l_z5_root_top3d_v002.tscn</x:v>
+      </x:c>
+      <x:c r="P282" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/source/env_base99_modular_room/env_base99_modular_room_assets_clean_v002.blend</x:v>
+      </x:c>
+      <x:c r="Q282" s="136" t="str">
+        <x:v>L梯; 连续坡面; 扶手</x:v>
+      </x:c>
+      <x:c r="R282" s="136" t="str">
+        <x:f>TEXTJOIN("|",TRUE,C282,D282,E282,F282,H282,I282)</x:f>
+        <x:v>场景|environment_module|base99_stair_l_z5|stair|俯视3D|default</x:v>
+      </x:c>
+      <x:c r="S282" s="136" t="str">
+        <x:f>IF(COUNTIF($R$6:$R$400,R282)&gt;1,"重复","唯一")</x:f>
+        <x:v>唯一</x:v>
+      </x:c>
+      <x:c r="T282" s="136"/>
+      <x:c r="U282" s="136" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="V282" s="137" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="W282" s="136" t="str">
+        <x:v>用户自制/项目内资产</x:v>
+      </x:c>
+      <x:c r="X282" s="136" t="str">
+        <x:v>2026-08-20：本轮基地系统、角色母版与资产流程登记。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="283" ht="66" customHeight="1">
+      <x:c r="A283" s="136" t="str">
+        <x:v>ENV-BASE99-STAIR-EXTERIOR-H4</x:v>
+      </x:c>
+      <x:c r="B283" s="136" t="str">
+        <x:v>基地99至100层4米外梯</x:v>
+      </x:c>
+      <x:c r="C283" s="136" t="str">
+        <x:v>场景</x:v>
+      </x:c>
+      <x:c r="D283" s="136" t="str">
+        <x:v>environment_module</x:v>
+      </x:c>
+      <x:c r="E283" s="136" t="str">
+        <x:v>base99_stair_exterior_h4</x:v>
+      </x:c>
+      <x:c r="F283" s="136" t="str">
+        <x:v>stair_exterior</x:v>
+      </x:c>
+      <x:c r="G283" s="136" t="str">
+        <x:v>ENV-BASE99-MODULAR-ROOM</x:v>
+      </x:c>
+      <x:c r="H283" s="136" t="str">
+        <x:v>俯视3D</x:v>
+      </x:c>
+      <x:c r="I283" s="136" t="str">
+        <x:v>default</x:v>
+      </x:c>
+      <x:c r="J283" s="136" t="str">
+        <x:v>基地99F/100F</x:v>
+      </x:c>
+      <x:c r="K283" s="136" t="str">
+        <x:v>正式美术已接入</x:v>
+      </x:c>
+      <x:c r="L283" s="136" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="M283" s="136" t="str">
+        <x:v>v002</x:v>
+      </x:c>
+      <x:c r="N283" s="136" t="str">
+        <x:v>5→9m；8.515m包络</x:v>
+      </x:c>
+      <x:c r="O283" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/runtime/env_base99_stair_exterior_h4/env_base99_stair_exterior_h4_root_top3d_v002.tscn</x:v>
+      </x:c>
+      <x:c r="P283" s="136" t="str">
+        <x:v>assets/art/environments/base_facility_3d/source/env_base99_modular_room/env_base99_modular_room_assets_clean_v002.blend</x:v>
+      </x:c>
+      <x:c r="Q283" s="136" t="str">
+        <x:v>外梯; H4; 连续坡面</x:v>
+      </x:c>
+      <x:c r="R283" s="136" t="str">
+        <x:f>TEXTJOIN("|",TRUE,C283,D283,E283,F283,H283,I283)</x:f>
+        <x:v>场景|environment_module|base99_stair_exterior_h4|stair_exterior|俯视3D|default</x:v>
+      </x:c>
+      <x:c r="S283" s="136" t="str">
+        <x:f>IF(COUNTIF($R$6:$R$400,R283)&gt;1,"重复","唯一")</x:f>
+        <x:v>唯一</x:v>
+      </x:c>
+      <x:c r="T283" s="136"/>
+      <x:c r="U283" s="136" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="V283" s="137" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="W283" s="136" t="str">
+        <x:v>用户自制/项目内资产</x:v>
+      </x:c>
+      <x:c r="X283" s="136" t="str">
+        <x:v>2026-08-20：本轮基地系统、角色母版与资产流程登记。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="284" ht="66" customHeight="1">
+      <x:c r="A284" s="136" t="str">
+        <x:v>PRP-BASE-RECOVERY-STATION-3D</x:v>
+      </x:c>
+      <x:c r="B284" s="136" t="str">
+        <x:v>基地状态恢复舱</x:v>
+      </x:c>
+      <x:c r="C284" s="136" t="str">
+        <x:v>设施</x:v>
+      </x:c>
+      <x:c r="D284" s="136" t="str">
+        <x:v>base_facility</x:v>
+      </x:c>
+      <x:c r="E284" s="136" t="str">
+        <x:v>base_recovery</x:v>
+      </x:c>
+      <x:c r="F284" s="136" t="str">
+        <x:v>root</x:v>
+      </x:c>
+      <x:c r="G284" s="136"/>
+      <x:c r="H284" s="136" t="str">
+        <x:v>俯视3D</x:v>
+      </x:c>
+      <x:c r="I284" s="136" t="str">
+        <x:v>default</x:v>
+      </x:c>
+      <x:c r="J284" s="136" t="str">
+        <x:v>主基地/99F</x:v>
+      </x:c>
+      <x:c r="K284" s="136" t="str">
+        <x:v>功能已接入</x:v>
+      </x:c>
+      <x:c r="L284" s="136" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="M284" s="136" t="str">
+        <x:v>v001</x:v>
+      </x:c>
+      <x:c r="N284" s="136" t="str">
+        <x:v>根缩放1</x:v>
+      </x:c>
+      <x:c r="O284" s="136" t="str">
+        <x:v>assets/art/props/base_world_3d/runtime/recovery_station/prp_base_recovery_station_root_top3d_v001.tscn</x:v>
+      </x:c>
+      <x:c r="P284" s="136" t="str">
+        <x:v>src/ui/BaseRecoveryMenu.gd; src/base/BaseEnergyService.gd</x:v>
+      </x:c>
+      <x:c r="Q284" s="136" t="str">
+        <x:v>恢复舱; HP; 手电; 基地能源</x:v>
+      </x:c>
+      <x:c r="R284" s="136" t="str">
+        <x:f>TEXTJOIN("|",TRUE,C284,D284,E284,F284,H284,I284)</x:f>
+        <x:v>设施|base_facility|base_recovery|root|俯视3D|default</x:v>
+      </x:c>
+      <x:c r="S284" s="136" t="str">
+        <x:f>IF(COUNTIF($R$6:$R$400,R284)&gt;1,"重复","唯一")</x:f>
+        <x:v>唯一</x:v>
+      </x:c>
+      <x:c r="T284" s="136"/>
+      <x:c r="U284" s="136" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="V284" s="137" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="W284" s="136" t="str">
+        <x:v>用户自制/项目内资产</x:v>
+      </x:c>
+      <x:c r="X284" s="136" t="str">
+        <x:v>2026-08-20：本轮基地系统、角色母版与资产流程登记。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="285" ht="66" customHeight="1">
+      <x:c r="A285" s="136" t="str">
+        <x:v>PRP-BASE-AVATAR-WARDROBE-001</x:v>
+      </x:c>
+      <x:c r="B285" s="136" t="str">
+        <x:v>基地角色衣柜</x:v>
+      </x:c>
+      <x:c r="C285" s="136" t="str">
+        <x:v>设施</x:v>
+      </x:c>
+      <x:c r="D285" s="136" t="str">
+        <x:v>base_facility</x:v>
+      </x:c>
+      <x:c r="E285" s="136" t="str">
+        <x:v>avatar_wardrobe</x:v>
+      </x:c>
+      <x:c r="F285" s="136" t="str">
+        <x:v>root</x:v>
+      </x:c>
+      <x:c r="G285" s="136"/>
+      <x:c r="H285" s="136" t="str">
+        <x:v>俯视3D</x:v>
+      </x:c>
+      <x:c r="I285" s="136" t="str">
+        <x:v>default</x:v>
+      </x:c>
+      <x:c r="J285" s="136" t="str">
+        <x:v>主基地/99F</x:v>
+      </x:c>
+      <x:c r="K285" s="136" t="str">
+        <x:v>功能已接入/复用模型</x:v>
+      </x:c>
+      <x:c r="L285" s="136" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="M285" s="136" t="str">
+        <x:v>v001</x:v>
+      </x:c>
+      <x:c r="N285" s="136" t="str">
+        <x:v>根缩放1</x:v>
+      </x:c>
+      <x:c r="O285" s="136" t="str">
+        <x:v>assets/art/props/base_world_3d/runtime/avatar_wardrobe/prp_base_avatar_wardrobe_root_top3d_v001.tscn</x:v>
+      </x:c>
+      <x:c r="P285" s="136" t="str">
+        <x:v>src/ui/wardrobe/WardrobeMenu3D.gd</x:v>
+      </x:c>
+      <x:c r="Q285" s="136" t="str">
+        <x:v>衣柜; avatar; 换装; 6分类</x:v>
+      </x:c>
+      <x:c r="R285" s="136" t="str">
+        <x:f>TEXTJOIN("|",TRUE,C285,D285,E285,F285,H285,I285)</x:f>
+        <x:v>设施|base_facility|avatar_wardrobe|root|俯视3D|default</x:v>
+      </x:c>
+      <x:c r="S285" s="136" t="str">
+        <x:f>IF(COUNTIF($R$6:$R$400,R285)&gt;1,"重复","唯一")</x:f>
+        <x:v>唯一</x:v>
+      </x:c>
+      <x:c r="T285" s="136"/>
+      <x:c r="U285" s="136" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="V285" s="137" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="W285" s="136" t="str">
+        <x:v>用户自制/项目内资产</x:v>
+      </x:c>
+      <x:c r="X285" s="136" t="str">
+        <x:v>2026-08-20：本轮基地系统、角色母版与资产流程登记。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="286" ht="66" customHeight="1">
+      <x:c r="A286" s="136" t="str">
+        <x:v>CHR-PLAYER-AVATAR-TEMPLATE-001</x:v>
+      </x:c>
+      <x:c r="B286" s="136" t="str">
+        <x:v>玩家角色1.5米制作母版</x:v>
+      </x:c>
+      <x:c r="C286" s="136" t="str">
+        <x:v>角色</x:v>
+      </x:c>
+      <x:c r="D286" s="136" t="str">
+        <x:v>authoring_template</x:v>
+      </x:c>
+      <x:c r="E286" s="136" t="str">
+        <x:v>player_avatar_template</x:v>
+      </x:c>
+      <x:c r="F286" s="136" t="str">
+        <x:v>root</x:v>
+      </x:c>
+      <x:c r="G286" s="136" t="str">
+        <x:v>CHR-PLY-CAPSULE01</x:v>
+      </x:c>
+      <x:c r="H286" s="136" t="str">
+        <x:v>全向3D</x:v>
+      </x:c>
+      <x:c r="I286" s="136" t="str">
+        <x:v>template</x:v>
+      </x:c>
+      <x:c r="J286" s="136" t="str">
+        <x:v>角色制作</x:v>
+      </x:c>
+      <x:c r="K286" s="136" t="str">
+        <x:v>正式制作母版</x:v>
+      </x:c>
+      <x:c r="L286" s="136" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="M286" s="136" t="str">
+        <x:v>v001</x:v>
+      </x:c>
+      <x:c r="N286" s="136" t="str">
+        <x:v>1.50m；根缩放1</x:v>
+      </x:c>
+      <x:c r="O286" s="136" t="str">
+        <x:v>assets/art/characters/player/chr_player_avatar_template_3d/source/chr_player_avatar_template_source_v001.blend</x:v>
+      </x:c>
+      <x:c r="P286" s="136" t="str">
+        <x:v>scripts/blender/validate_player_avatar_asset_template.py</x:v>
+      </x:c>
+      <x:c r="Q286" s="136" t="str">
+        <x:v>角色母版; 1.5米; 挂点; 配件</x:v>
+      </x:c>
+      <x:c r="R286" s="136" t="str">
+        <x:f>TEXTJOIN("|",TRUE,C286,D286,E286,F286,H286,I286)</x:f>
+        <x:v>角色|authoring_template|player_avatar_template|root|全向3D|template</x:v>
+      </x:c>
+      <x:c r="S286" s="136" t="str">
+        <x:f>IF(COUNTIF($R$6:$R$400,R286)&gt;1,"重复","唯一")</x:f>
+        <x:v>唯一</x:v>
+      </x:c>
+      <x:c r="T286" s="136"/>
+      <x:c r="U286" s="136" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="V286" s="137" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="W286" s="136" t="str">
+        <x:v>用户自制/项目内资产</x:v>
+      </x:c>
+      <x:c r="X286" s="136" t="str">
+        <x:v>2026-08-20：本轮基地系统、角色母版与资产流程登记。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:X2"/>
@@ -36863,7 +37866,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R312686a395b54d32"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc90492b8a87c477b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43698,13 +44701,27 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="78" customHeight="1">
-      <x:c r="A23" s="136"/>
-      <x:c r="B23" s="136"/>
-      <x:c r="C23" s="136"/>
-      <x:c r="D23" s="136"/>
-      <x:c r="E23" s="136"/>
-      <x:c r="F23" s="136"/>
-      <x:c r="G23" s="136"/>
+      <x:c r="A23" s="136" t="str">
+        <x:v>v0.1.19</x:v>
+      </x:c>
+      <x:c r="B23" s="137" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="C23" s="136" t="str">
+        <x:v>基地系统/时间/Avatar/3D流程收口</x:v>
+      </x:c>
+      <x:c r="D23" s="136" t="str">
+        <x:v>6项资产/3项Skill/5米结构/11设施</x:v>
+      </x:c>
+      <x:c r="E23" s="136" t="str">
+        <x:v>平台改为5米并联动两类楼梯与栏杆碰撞；新增物理楼层权威、时间日夜、基地能源恢复舱、主页面、衣柜、脱困和1.5米角色母版。</x:v>
+      </x:c>
+      <x:c r="F23" s="136" t="str">
+        <x:v>视觉替换不改变原门、设施、玩家碰撞和战斗脚本；旧Z7/H2资产保留回滚；新Skill草稿未安装。</x:v>
+      </x:c>
+      <x:c r="G23" s="136" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="100" customHeight="1">
       <x:c r="A24" s="136"/>
@@ -43966,16 +44983,16 @@
         <x:v>3D-场景通用</x:v>
       </x:c>
       <x:c r="C5" s="277" t="n">
-        <x:v>52</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D5" s="277" t="n">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E5" s="277" t="n">
-        <x:v>52</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="F5" s="277" t="n">
-        <x:v>36</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="G5" s="278" t="str">
         <x:v>关卡结构、地板、墙体、走廊、楼梯、楼板与环境套件</x:v>
@@ -43999,16 +45016,16 @@
         <x:v>3D-设施</x:v>
       </x:c>
       <x:c r="C6" s="280" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D6" s="280" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E6" s="280" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F6" s="280" t="n">
         <x:v>15</x:v>
-      </x:c>
-      <x:c r="D6" s="280" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E6" s="280" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F6" s="280" t="n">
-        <x:v>13</x:v>
       </x:c>
       <x:c r="G6" s="281" t="str">
         <x:v>门扇、灯具、开关、终端、工作台、储物与服务设施</x:v>
@@ -44069,19 +45086,15 @@
         <x:v>3D-角色</x:v>
       </x:c>
       <x:c r="C8" s="280" t="n">
-        <x:f>COUNTA('3D-角色'!$A$5:$A$204)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D8" s="280" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="280" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D8" s="280" t="n">
-        <x:f>COUNTIF('3D-角色'!$D$5:$D$204,"&lt;&gt;")</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E8" s="280" t="n">
-        <x:f>COUNTIF('3D-角色'!$G$5:$G$204,"&lt;&gt;")</x:f>
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="F8" s="280" t="n">
-        <x:f>COUNTIF('3D-角色'!$H$5:$H$204,"开")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="G8" s="281" t="str">
@@ -44291,19 +45304,19 @@
         <x:v>9个分类分页</x:v>
       </x:c>
       <x:c r="C14" s="315" t="n">
-        <x:v>99</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D14" s="315" t="n">
-        <x:v>37</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E14" s="315" t="n">
-        <x:v>96</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="F14" s="315" t="n">
-        <x:v>53</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="G14" s="316" t="str">
-        <x:v>更新日期：2026-08-18；基地100层上层围护与18米封顶接入</x:v>
+        <x:v>更新日期：2026-08-20；5米基地结构、恢复舱、衣柜与角色母版接入</x:v>
       </x:c>
       <x:c r="H14" s="136"/>
       <x:c r="I14" s="136"/>

</xml_diff>